<commit_message>
Update Baseline & Concurrency Load Test specs and report Excel
</commit_message>
<xml_diff>
--- a/load-tests/load_test_report.xlsx
+++ b/load-tests/load_test_report.xlsx
@@ -29,7 +29,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00263238"/>
+      <color rgb="001B365D"/>
       <sz val="16"/>
     </font>
     <font>
@@ -57,8 +57,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0037474F"/>
-        <bgColor rgb="0037474F"/>
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
       </patternFill>
     </fill>
     <fill>
@@ -69,8 +69,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00455A64"/>
-        <bgColor rgb="00455A64"/>
+        <fgColor rgb="002E5B88"/>
+        <bgColor rgb="002E5B88"/>
       </patternFill>
     </fill>
   </fills>
@@ -487,7 +487,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -496,7 +496,7 @@
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CookSmart API Baseline Performance &amp; 100 Virtual Users Load Test Report</t>
+          <t>CookSmart API Baseline &amp; Concurrency Load Test Report (100 Virtual Users)</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Simulated Virtual Users (VU)</t>
+          <t>Virtual Users (Concurrent Threads)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>&lt; 300 ms</t>
+          <t>&lt; 250 ms</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Host CPU &amp; Memory</t>
+          <t>Host CPU &amp; Memory Usage</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">

</xml_diff>